<commit_message>
Add notificaciones cese app and improve launcher flow
</commit_message>
<xml_diff>
--- a/derechosTransmision/templates/acta_data.xlsx
+++ b/derechosTransmision/templates/acta_data.xlsx
@@ -541,12 +541,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -689,14 +689,31 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>canal tv</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TUDN o ESPN. Deje este campo en blanco si no se especifica el canal</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>hora fin diligencia</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr"/>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr"/>
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>dos de la tarde con dos minutos</t>
         </is>
@@ -709,6 +726,6 @@
     <mergeCell ref="A3:C3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <legacyDrawing ns1:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>